<commit_message>
Added reference threshold sensitivity analysis via RDA. It refactored the stage 1 and RDA in a new way.
</commit_message>
<xml_diff>
--- a/results/01_pollution_assessment/tables/pc_loadings.xlsx
+++ b/results/01_pollution_assessment/tables/pc_loadings.xlsx
@@ -462,19 +462,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3606101831871588</v>
+        <v>0.8702291985393624</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1877290339865944</v>
+        <v>0.2379641446746292</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1119599705742961</v>
+        <v>-0.07105278801769738</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3202135299974001</v>
+        <v>-0.1827130022512433</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.06073174242921327</v>
+        <v>-0.1581838477524132</v>
       </c>
     </row>
     <row r="3">
@@ -484,19 +484,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.5214695814339583</v>
+        <v>0.7516662796993644</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1832330240339628</v>
+        <v>0.4159269540841169</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3068722930964033</v>
+        <v>-0.009669201241349188</v>
       </c>
       <c r="E3" t="n">
-        <v>0.7292323415583598</v>
+        <v>-0.3428887083211319</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.05202754895816125</v>
+        <v>-0.1669763089373493</v>
       </c>
     </row>
     <row r="4">
@@ -506,19 +506,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4094264607169094</v>
+        <v>0.7037991818052765</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9272058070250112</v>
+        <v>0.1342316645090597</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.04979837077098496</v>
+        <v>-0.2738314766945599</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2056390972923768</v>
+        <v>0.5031894760773989</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.2132220398666368</v>
+        <v>-0.04290576823452369</v>
       </c>
     </row>
     <row r="5">
@@ -528,19 +528,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.06507095861101514</v>
+        <v>0.5151483306417299</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2746698837258384</v>
+        <v>0.7317658414115079</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3508990558530958</v>
+        <v>0.1921967033167705</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3814571777589376</v>
+        <v>-0.01971383312066507</v>
       </c>
       <c r="F5" t="n">
-        <v>0.06571909405534154</v>
+        <v>0.02147117793593797</v>
       </c>
     </row>
     <row r="6">
@@ -550,19 +550,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.5073370775090991</v>
+        <v>0.5849815933099674</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3433756328793434</v>
+        <v>0.2288326968670686</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1304823760386074</v>
+        <v>-0.1253045030851519</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6099595439975646</v>
+        <v>-0.2110975536903878</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7153959372751683</v>
+        <v>-0.02605531144045951</v>
       </c>
     </row>
     <row r="7">
@@ -572,19 +572,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.6719704293106613</v>
+        <v>0.9236859568955842</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5670885411507882</v>
+        <v>0.05851055499934814</v>
       </c>
       <c r="D7" t="n">
-        <v>0.106670535502527</v>
+        <v>-0.1303087435244772</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3577982473586992</v>
+        <v>0.1397499600016423</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.2422077762230097</v>
+        <v>-0.2077635501025502</v>
       </c>
     </row>
     <row r="8">
@@ -594,19 +594,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.7543749497540863</v>
+        <v>0.8508569920196865</v>
       </c>
       <c r="C8" t="n">
-        <v>0.6971553913821574</v>
+        <v>0.1002996207337038</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1474068558952266</v>
+        <v>-0.1394899566632955</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4925226869386944</v>
+        <v>0.1404083500871058</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.4369477504943916</v>
+        <v>-0.258034181786378</v>
       </c>
     </row>
     <row r="9">
@@ -616,19 +616,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5.107143789904225</v>
+        <v>0.7568136738017586</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.6096427455103576</v>
+        <v>-0.475517059753405</v>
       </c>
       <c r="D9" t="n">
-        <v>0.07425475450888282</v>
+        <v>0.06445292489375971</v>
       </c>
       <c r="E9" t="n">
-        <v>0.183992574608914</v>
+        <v>-0.4162016518169434</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.01137937574588698</v>
+        <v>0.03772586532141763</v>
       </c>
     </row>
     <row r="10">
@@ -638,19 +638,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.1038857224785213</v>
+        <v>0.1492387911722579</v>
       </c>
       <c r="C10" t="n">
-        <v>0.4042564135127725</v>
+        <v>0.2206785018871727</v>
       </c>
       <c r="D10" t="n">
-        <v>1.473122055190723</v>
+        <v>0.8421663524838221</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.4778803022358065</v>
+        <v>0.391581521956009</v>
       </c>
       <c r="F10" t="n">
-        <v>0.02409371635469992</v>
+        <v>0.07670048978478905</v>
       </c>
     </row>
     <row r="11">
@@ -660,19 +660,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-2.335244129682883</v>
+        <v>-0.5552484960147785</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7543773998348152</v>
+        <v>0.6671581283034471</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2227753496080398</v>
+        <v>-0.0813582673073638</v>
       </c>
       <c r="E11" t="n">
-        <v>0.4044778329318201</v>
+        <v>0.4501981861406558</v>
       </c>
       <c r="F11" t="n">
-        <v>0.01610606886892633</v>
+        <v>-0.08022077880775023</v>
       </c>
     </row>
     <row r="12">
@@ -682,19 +682,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.682317074569096</v>
+        <v>0.7161461618296157</v>
       </c>
       <c r="C12" t="n">
-        <v>1.711686459665509</v>
+        <v>-0.3676552722118935</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.5485684584588472</v>
+        <v>-0.2155960307069405</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.7048118292085341</v>
+        <v>0.3797318632058666</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1614578467457171</v>
+        <v>0.191464099829989</v>
       </c>
     </row>
     <row r="13">
@@ -704,19 +704,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.3997005489335929</v>
+        <v>0.7956417771140938</v>
       </c>
       <c r="C13" t="n">
-        <v>0.2211779878078544</v>
+        <v>-0.2105025932620872</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1854150206582691</v>
+        <v>0.2935612617016572</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.06578916343869991</v>
+        <v>0.2001884790675518</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.04718811875168219</v>
+        <v>0.06886790650655654</v>
       </c>
     </row>
     <row r="14">
@@ -726,19 +726,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.03956333063927631</v>
+        <v>0.1622513922330454</v>
       </c>
       <c r="C14" t="n">
-        <v>0.1869113238801454</v>
+        <v>0.2444577607301594</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.03677150855389216</v>
+        <v>-0.1962156393246558</v>
       </c>
       <c r="E14" t="n">
-        <v>0.05473297279913972</v>
+        <v>0.01458086909026485</v>
       </c>
       <c r="F14" t="n">
-        <v>0.3936352260306018</v>
+        <v>0.8372685141895162</v>
       </c>
     </row>
     <row r="15">
@@ -748,19 +748,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.6317417252198432</v>
+        <v>0.6540105406045499</v>
       </c>
       <c r="C15" t="n">
-        <v>0.5112024472909085</v>
+        <v>-0.3578965853786691</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.2180187387240261</v>
+        <v>-0.2471796404340765</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.1479949182682809</v>
+        <v>0.2808305309241664</v>
       </c>
       <c r="F15" t="n">
-        <v>0.03411852705251382</v>
+        <v>0.1779647265487449</v>
       </c>
     </row>
     <row r="16">
@@ -770,19 +770,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.8038463549921078</v>
+        <v>0.5114263489382381</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.04268633717272017</v>
+        <v>-0.2072619187901369</v>
       </c>
       <c r="D16" t="n">
-        <v>1.01681817994705</v>
+        <v>0.770708187586743</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.3993110320221156</v>
+        <v>-0.07578910028212038</v>
       </c>
       <c r="F16" t="n">
-        <v>0.05105283293193173</v>
+        <v>0.1099886831713247</v>
       </c>
     </row>
     <row r="17">
@@ -792,19 +792,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.1557326474084392</v>
+        <v>0.3541510935229762</v>
       </c>
       <c r="C17" t="n">
-        <v>0.07203148140934948</v>
+        <v>0.463517538084968</v>
       </c>
       <c r="D17" t="n">
-        <v>0.08152911706652521</v>
+        <v>-0.06864382451046237</v>
       </c>
       <c r="E17" t="n">
-        <v>0.3426865634316861</v>
+        <v>-0.3509417745051812</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1848546464642934</v>
+        <v>0.3503087775069246</v>
       </c>
     </row>
     <row r="18">
@@ -822,19 +822,19 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>37.45996204980186</v>
+        <v>6.892655394744991</v>
       </c>
       <c r="C19" t="n">
-        <v>6.31573003109829</v>
+        <v>2.194022211947241</v>
       </c>
       <c r="D19" t="n">
-        <v>3.932436519405018</v>
+        <v>1.720183089762909</v>
       </c>
       <c r="E19" t="n">
-        <v>2.793457029766627</v>
+        <v>1.409844255664912</v>
       </c>
       <c r="F19" t="n">
-        <v>1.039712293364102</v>
+        <v>1.088277973084644</v>
       </c>
     </row>
     <row r="20">
@@ -844,19 +844,19 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.6864431839375965</v>
+        <v>0.4307909621715619</v>
       </c>
       <c r="C20" t="n">
-        <v>0.115733962188046</v>
+        <v>0.1371263882467026</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0720607842961533</v>
+        <v>0.1075114431101818</v>
       </c>
       <c r="E20" t="n">
-        <v>0.05118930807128268</v>
+        <v>0.08811526597905699</v>
       </c>
       <c r="F20" t="n">
-        <v>0.01905243299731773</v>
+        <v>0.06801737331779023</v>
       </c>
     </row>
     <row r="21">
@@ -866,19 +866,19 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.6864431839375965</v>
+        <v>0.4307909621715619</v>
       </c>
       <c r="C21" t="n">
-        <v>0.8021771461256425</v>
+        <v>0.5679173504182645</v>
       </c>
       <c r="D21" t="n">
-        <v>0.8742379304217958</v>
+        <v>0.6754287935284463</v>
       </c>
       <c r="E21" t="n">
-        <v>0.9254272384930784</v>
+        <v>0.7635440595075033</v>
       </c>
       <c r="F21" t="n">
-        <v>0.9444796714903961</v>
+        <v>0.8315614328252935</v>
       </c>
     </row>
   </sheetData>

</xml_diff>